<commit_message>
create multiple docotors/patients, add bulk delete
</commit_message>
<xml_diff>
--- a/seeders/doctors_sample_data.xlsx
+++ b/seeders/doctors_sample_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="106">
   <si>
     <t>name</t>
   </si>
@@ -128,6 +128,210 @@
   </si>
   <si>
     <t>B+</t>
+  </si>
+  <si>
+    <t>Dr. Layla Hassan</t>
+  </si>
+  <si>
+    <t>lhassan@tiryaq.com</t>
+  </si>
+  <si>
+    <t>1985-08-22</t>
+  </si>
+  <si>
+    <t>female</t>
+  </si>
+  <si>
+    <t>+974 5523 2222</t>
+  </si>
+  <si>
+    <t>29823456789</t>
+  </si>
+  <si>
+    <t>Consultant</t>
+  </si>
+  <si>
+    <t>Daman Healthcare</t>
+  </si>
+  <si>
+    <t>Neurology</t>
+  </si>
+  <si>
+    <t>Brain and Nerve</t>
+  </si>
+  <si>
+    <t>2013-03-15</t>
+  </si>
+  <si>
+    <t>Expert in epilepsy and movement disorders</t>
+  </si>
+  <si>
+    <t>PhD</t>
+  </si>
+  <si>
+    <t>MON,TUE,WED,THU,FRI</t>
+  </si>
+  <si>
+    <t>09:00</t>
+  </si>
+  <si>
+    <t>17:00</t>
+  </si>
+  <si>
+    <t>O+</t>
+  </si>
+  <si>
+    <t>Dr. Youssef Khalil</t>
+  </si>
+  <si>
+    <t>ykhalil@tiryaq.com</t>
+  </si>
+  <si>
+    <t>1990-12-03</t>
+  </si>
+  <si>
+    <t>+974 5534 3333</t>
+  </si>
+  <si>
+    <t>30034567890</t>
+  </si>
+  <si>
+    <t>Specialist</t>
+  </si>
+  <si>
+    <t>Seha Health Insurance</t>
+  </si>
+  <si>
+    <t>Orthopedics</t>
+  </si>
+  <si>
+    <t>Bone and Joint</t>
+  </si>
+  <si>
+    <t>junior</t>
+  </si>
+  <si>
+    <t>2018-06-01</t>
+  </si>
+  <si>
+    <t>Focus on sports injuries and joint reconstruction</t>
+  </si>
+  <si>
+    <t>MBBS</t>
+  </si>
+  <si>
+    <t>TUE,WED,THU,FRI</t>
+  </si>
+  <si>
+    <t>07:00</t>
+  </si>
+  <si>
+    <t>15:00</t>
+  </si>
+  <si>
+    <t>A+</t>
+  </si>
+  <si>
+    <t>Dr. Mariam Saleh</t>
+  </si>
+  <si>
+    <t>msaleh@tiryaq.com</t>
+  </si>
+  <si>
+    <t>1978-06-17</t>
+  </si>
+  <si>
+    <t>+974 5545 4444</t>
+  </si>
+  <si>
+    <t>29945678901</t>
+  </si>
+  <si>
+    <t>Associate Consultant</t>
+  </si>
+  <si>
+    <t>Qatar General Insurance</t>
+  </si>
+  <si>
+    <t>Dermatology</t>
+  </si>
+  <si>
+    <t>Skin and Aesthetics</t>
+  </si>
+  <si>
+    <t>associate</t>
+  </si>
+  <si>
+    <t>2008-11-20</t>
+  </si>
+  <si>
+    <t>Specialist in cosmetic dermatology and skin cancer screening</t>
+  </si>
+  <si>
+    <t>MON,WED,FRI</t>
+  </si>
+  <si>
+    <t>10:00</t>
+  </si>
+  <si>
+    <t>18:00</t>
+  </si>
+  <si>
+    <t>AB-</t>
+  </si>
+  <si>
+    <t>Dr. Bob Smith</t>
+  </si>
+  <si>
+    <t>bsmith@tiryaq.com</t>
+  </si>
+  <si>
+    <t>+974 5545 4443</t>
+  </si>
+  <si>
+    <t>Dr. Tariq Al-Zaabi</t>
+  </si>
+  <si>
+    <t>1987-02-28</t>
+  </si>
+  <si>
+    <t>+974 5556 5555</t>
+  </si>
+  <si>
+    <t>31056789012</t>
+  </si>
+  <si>
+    <t>Junior Consultant</t>
+  </si>
+  <si>
+    <t>Al Koot Insurance</t>
+  </si>
+  <si>
+    <t>General Surgery</t>
+  </si>
+  <si>
+    <t>Surgery</t>
+  </si>
+  <si>
+    <t>2016-04-10</t>
+  </si>
+  <si>
+    <t>Laparoscopic and robotic surgery specialist</t>
+  </si>
+  <si>
+    <t>Fellowship</t>
+  </si>
+  <si>
+    <t>MON,TUE,THU,FRI</t>
+  </si>
+  <si>
+    <t>06:00</t>
+  </si>
+  <si>
+    <t>14:00</t>
+  </si>
+  <si>
+    <t>O-</t>
   </si>
 </sst>
 </file>
@@ -177,7 +381,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -187,6 +391,9 @@
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -496,29 +703,29 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:T7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="21.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="4" width="18.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="4" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="4" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="4" width="50.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="4" width="55.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="4" width="35.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="4" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="21.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="18.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="5" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="6" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="6" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="5" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="5" width="55.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="5" width="35.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="5" width="10.862142857142858" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -645,6 +852,316 @@
         <v>37</v>
       </c>
     </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="M3" s="3">
+        <v>14</v>
+      </c>
+      <c r="N3" s="3">
+        <v>8</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="M4" s="3">
+        <v>7</v>
+      </c>
+      <c r="N4" s="3">
+        <v>2</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="S4" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="M5" s="3">
+        <v>20</v>
+      </c>
+      <c r="N5" s="3">
+        <v>6</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="S5" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F6" s="4">
+        <v>29855520111</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="M6" s="3">
+        <v>20</v>
+      </c>
+      <c r="N6" s="3">
+        <v>6</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="T6" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="M7" s="3">
+        <v>9</v>
+      </c>
+      <c r="N7" s="3">
+        <v>9</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="R7" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="S7" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="T7" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: re-sync duty schedule now deletes and recreates calendar for guaranteed clean slate
</commit_message>
<xml_diff>
--- a/seeders/doctors_sample_data.xlsx
+++ b/seeders/doctors_sample_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
   <si>
     <t>name</t>
   </si>
@@ -176,150 +176,6 @@
   </si>
   <si>
     <t>O+</t>
-  </si>
-  <si>
-    <t>Dr. Youssef Khalil</t>
-  </si>
-  <si>
-    <t>ykhalil@tiryaq.com</t>
-  </si>
-  <si>
-    <t>1990-12-03</t>
-  </si>
-  <si>
-    <t>+974 5534 3333</t>
-  </si>
-  <si>
-    <t>Specialist</t>
-  </si>
-  <si>
-    <t>Seha Health Insurance</t>
-  </si>
-  <si>
-    <t>Orthopedics</t>
-  </si>
-  <si>
-    <t>Bone and Joint</t>
-  </si>
-  <si>
-    <t>junior</t>
-  </si>
-  <si>
-    <t>2018-06-01</t>
-  </si>
-  <si>
-    <t>Focus on sports injuries and joint reconstruction</t>
-  </si>
-  <si>
-    <t>MBBS</t>
-  </si>
-  <si>
-    <t>TUE,WED,THU,FRI</t>
-  </si>
-  <si>
-    <t>07:00</t>
-  </si>
-  <si>
-    <t>15:00</t>
-  </si>
-  <si>
-    <t>A+</t>
-  </si>
-  <si>
-    <t>Dr. Mariam Saleh</t>
-  </si>
-  <si>
-    <t>msaleh@tiryaq.com</t>
-  </si>
-  <si>
-    <t>1978-06-17</t>
-  </si>
-  <si>
-    <t>+974 5545 4444</t>
-  </si>
-  <si>
-    <t>Associate Consultant</t>
-  </si>
-  <si>
-    <t>Qatar General Insurance</t>
-  </si>
-  <si>
-    <t>Dermatology</t>
-  </si>
-  <si>
-    <t>Skin and Aesthetics</t>
-  </si>
-  <si>
-    <t>associate</t>
-  </si>
-  <si>
-    <t>2008-11-20</t>
-  </si>
-  <si>
-    <t>Specialist in cosmetic dermatology and skin cancer screening</t>
-  </si>
-  <si>
-    <t>MON,WED,FRI</t>
-  </si>
-  <si>
-    <t>10:00</t>
-  </si>
-  <si>
-    <t>18:00</t>
-  </si>
-  <si>
-    <t>AB-</t>
-  </si>
-  <si>
-    <t>Dr. Bob Smith</t>
-  </si>
-  <si>
-    <t>bsmith@tiryaq.com</t>
-  </si>
-  <si>
-    <t>+974 5545 4443</t>
-  </si>
-  <si>
-    <t>Dr. Tariq Al-Zaabi</t>
-  </si>
-  <si>
-    <t>1987-02-28</t>
-  </si>
-  <si>
-    <t>+974 5556 5555</t>
-  </si>
-  <si>
-    <t>Junior Consultant</t>
-  </si>
-  <si>
-    <t>Al Koot Insurance</t>
-  </si>
-  <si>
-    <t>General Surgery</t>
-  </si>
-  <si>
-    <t>Surgery</t>
-  </si>
-  <si>
-    <t>2016-04-10</t>
-  </si>
-  <si>
-    <t>Laparoscopic and robotic surgery specialist</t>
-  </si>
-  <si>
-    <t>Fellowship</t>
-  </si>
-  <si>
-    <t>MON,TUE,THU,FRI</t>
-  </si>
-  <si>
-    <t>06:00</t>
-  </si>
-  <si>
-    <t>14:00</t>
-  </si>
-  <si>
-    <t>O-</t>
   </si>
 </sst>
 </file>
@@ -381,18 +237,18 @@
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -700,33 +556,33 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="21.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="18.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="6" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="5" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="5" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="21.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="6" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="18.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="7" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="6" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="6" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="6" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="6" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="6" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="6" width="13.862142857142858" customWidth="1" bestFit="1"/>
     <col min="14" max="14" style="7" width="18.005" customWidth="1" bestFit="1"/>
     <col min="15" max="15" style="7" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="5" width="50.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="5" width="55.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="5" width="35.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="5" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="6" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="6" width="55.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="6" width="35.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="6" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="6" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="6" width="10.862142857142858" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -742,10 +598,10 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -766,10 +622,10 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="4" t="s">
         <v>14</v>
       </c>
       <c r="P1" s="1" t="s">
@@ -807,10 +663,10 @@
       <c r="E2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="5">
         <v>1</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="5">
         <v>28601234567</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -872,10 +728,10 @@
       <c r="E3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="5">
         <v>2</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="5">
         <v>29823456789</v>
       </c>
       <c r="H3" s="1" t="s">
@@ -919,266 +775,6 @@
       </c>
       <c r="U3" s="1" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F4" s="2">
-        <v>3</v>
-      </c>
-      <c r="G4" s="2">
-        <v>30034567890</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="N4" s="4">
-        <v>7</v>
-      </c>
-      <c r="O4" s="4">
-        <v>2</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="R4" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="S4" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="T4" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="U4" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
-      <c r="A5" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F5" s="2">
-        <v>4</v>
-      </c>
-      <c r="G5" s="2">
-        <v>29945678901</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="N5" s="4">
-        <v>20</v>
-      </c>
-      <c r="O5" s="4">
-        <v>6</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="R5" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="S5" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="T5" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="U5" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="F6" s="2">
-        <v>5</v>
-      </c>
-      <c r="G6" s="3">
-        <v>29855520111</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="N6" s="4">
-        <v>20</v>
-      </c>
-      <c r="O6" s="4">
-        <v>6</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="R6" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="S6" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="T6" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="F7" s="2">
-        <v>6</v>
-      </c>
-      <c r="G7" s="2">
-        <v>31056789012</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="N7" s="4">
-        <v>9</v>
-      </c>
-      <c r="O7" s="4">
-        <v>9</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="Q7" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="R7" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="S7" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="T7" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
testing and bug fixes
</commit_message>
<xml_diff>
--- a/seeders/doctors_sample_data.xlsx
+++ b/seeders/doctors_sample_data.xlsx
@@ -79,10 +79,10 @@
     <t>bloodGroup</t>
   </si>
   <si>
-    <t>Dr. Layla Hassan</t>
-  </si>
-  <si>
-    <t>lhassan@tiryaq.com</t>
+    <t>Dr. Sami Taha</t>
+  </si>
+  <si>
+    <t>staha@tiryaq.com</t>
   </si>
   <si>
     <t>1985-08-22</t>
@@ -91,7 +91,7 @@
     <t>female</t>
   </si>
   <si>
-    <t>+974 5523 2222</t>
+    <t>+974 5512 9999</t>
   </si>
   <si>
     <t>Consultant</t>
@@ -100,7 +100,7 @@
     <t>Daman Healthcare</t>
   </si>
   <si>
-    <t>Neurology</t>
+    <t>General (Adult) Internal Medicine</t>
   </si>
   <si>
     <t>Brain and Nerve</t>
@@ -135,19 +135,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -183,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -191,11 +185,8 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -508,27 +499,27 @@
   <dimension ref="A1:U2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="21.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="18.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="6" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="5" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="5" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="6" width="18.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="6" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="5" width="50.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="5" width="55.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="5" width="35.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="5" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="21.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="18.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="5" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="4" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="5" width="18.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="4" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="4" width="55.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="4" width="35.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="4" width="10.862142857142858" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -571,10 +562,10 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
       <c r="P1" s="1" t="s">
@@ -612,10 +603,10 @@
       <c r="E2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="2">
         <v>2</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="2">
         <v>29823456789</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -636,10 +627,10 @@
       <c r="M2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="N2" s="4">
+      <c r="N2" s="2">
         <v>14</v>
       </c>
-      <c r="O2" s="4">
+      <c r="O2" s="2">
         <v>8</v>
       </c>
       <c r="P2" s="1" t="s">

</xml_diff>

<commit_message>
doctor appointment change in workflow
</commit_message>
<xml_diff>
--- a/seeders/doctors_sample_data.xlsx
+++ b/seeders/doctors_sample_data.xlsx
@@ -79,10 +79,10 @@
     <t>bloodGroup</t>
   </si>
   <si>
-    <t>Dr. Sami Taha</t>
-  </si>
-  <si>
-    <t>staha@tiryaq.com</t>
+    <t>Dr. Sami Taha(doctor1)</t>
+  </si>
+  <si>
+    <t>doctor1@tiryaq.com</t>
   </si>
   <si>
     <t>1985-08-22</t>

</xml_diff>

<commit_message>
Calendar migration to Hospital table; remove hard-delete (patients+doctors); fix updatedAt-null GSI bug; JWT-enforce invoice scoping; CORS cleanup; cache-clean in deploy script
</commit_message>
<xml_diff>
--- a/seeders/doctors_sample_data.xlsx
+++ b/seeders/doctors_sample_data.xlsx
@@ -79,7 +79,7 @@
     <t>bloodGroup</t>
   </si>
   <si>
-    <t>Dr. Sami Taha(doctor1)</t>
+    <t>Dr. Omar Rashidi(doctor1)</t>
   </si>
   <si>
     <t>doctor1@tiryaq.com</t>
@@ -91,7 +91,7 @@
     <t>male</t>
   </si>
   <si>
-    <t>+974 5512 9999</t>
+    <t>+974 7878 9999</t>
   </si>
   <si>
     <t>Consultant</t>
@@ -607,7 +607,7 @@
         <v>2</v>
       </c>
       <c r="G2" s="2">
-        <v>29823456789</v>
+        <v>33445566777</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
user manual, data based on role, ui changes
</commit_message>
<xml_diff>
--- a/seeders/doctors_sample_data.xlsx
+++ b/seeders/doctors_sample_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="49">
   <si>
     <t>name</t>
   </si>
@@ -79,6 +79,58 @@
     <t>bloodGroup</t>
   </si>
   <si>
+    <t>Dr. Roula Mansour</t>
+  </si>
+  <si>
+    <t>doctor2@tiryaq.com</t>
+  </si>
+  <si>
+    <t>1975-01-30</t>
+  </si>
+  <si>
+    <t>female</t>
+  </si>
+  <si>
+    <t>+974 7878 8888</t>
+  </si>
+  <si>
+    <t>Clinic Advisor</t>
+  </si>
+  <si>
+    <t>Doha Insurance</t>
+  </si>
+  <si>
+    <t>Nerves</t>
+  </si>
+  <si>
+    <t>Brain and Nerve</t>
+  </si>
+  <si>
+    <t>junior</t>
+  </si>
+  <si>
+    <t>2013-03-15</t>
+  </si>
+  <si>
+    <t>Expert in epilepsy and movement disorders</t>
+  </si>
+  <si>
+    <t>PhD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WED,THU,SAT,SUN
+</t>
+  </si>
+  <si>
+    <t>09:00</t>
+  </si>
+  <si>
+    <t>17:00</t>
+  </si>
+  <si>
+    <t>A+</t>
+  </si>
+  <si>
     <t>Dr. Omar Rashidi(doctor1)</t>
   </si>
   <si>
@@ -103,28 +155,10 @@
     <t>General (Adult) Internal Medicine</t>
   </si>
   <si>
-    <t>Brain and Nerve</t>
-  </si>
-  <si>
     <t>senior</t>
   </si>
   <si>
-    <t>2013-03-15</t>
-  </si>
-  <si>
-    <t>Expert in epilepsy and movement disorders</t>
-  </si>
-  <si>
-    <t>PhD</t>
-  </si>
-  <si>
     <t>MON,TUE,WED,THU,FRI</t>
-  </si>
-  <si>
-    <t>09:00</t>
-  </si>
-  <si>
-    <t>17:00</t>
   </si>
   <si>
     <t>O+</t>
@@ -177,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -187,6 +221,9 @@
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -496,30 +533,30 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="4" width="21.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="4" width="18.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="5" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="4" width="25.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="4" width="20.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="4" width="13.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="5" width="18.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="4" width="50.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="4" width="55.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="4" width="35.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="4" width="12.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="4" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="21.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="10.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="18.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="6" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="25.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="5" width="20.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="5" width="13.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="6" width="18.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="6" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="5" width="50.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="5" width="55.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="5" width="35.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="5" width="12.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="5" width="10.862142857142858" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -587,7 +624,7 @@
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
@@ -603,11 +640,11 @@
       <c r="E2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="2">
-        <v>2</v>
-      </c>
-      <c r="G2" s="2">
-        <v>33445566777</v>
+      <c r="F2" s="4">
+        <v>1</v>
+      </c>
+      <c r="G2" s="4">
+        <v>89896932351</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>26</v>
@@ -650,6 +687,71 @@
       </c>
       <c r="U2" s="1" t="s">
         <v>37</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+      <c r="A3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" s="2">
+        <v>2</v>
+      </c>
+      <c r="G3" s="2">
+        <v>33445566777</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N3" s="2">
+        <v>14</v>
+      </c>
+      <c r="O3" s="2">
+        <v>8</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(appointments): refresh doctors/patients on opening New Appointment if lists are empty
</commit_message>
<xml_diff>
--- a/seeders/doctors_sample_data.xlsx
+++ b/seeders/doctors_sample_data.xlsx
@@ -131,7 +131,7 @@
     <t>A+</t>
   </si>
   <si>
-    <t>Dr. Omar Rashidi(doctor1)</t>
+    <t>Dr. Omar Rashidi</t>
   </si>
   <si>
     <t>doctor1@tiryaq.com</t>
@@ -169,7 +169,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -180,6 +180,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -222,7 +228,7 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -624,7 +630,7 @@
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>

</xml_diff>